<commit_message>
Update num.txt | 2026-08-05 08:20:57 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="114">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,30 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第654回</t>
+  </si>
+  <si>
+    <t>2026年8月5日（令和8年8月5日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１医療機器の保険適用について
+２医薬品の新規薬価収載等について
+３再生医療等製品の保険適用について
+４最適使用推進ガイドラインについて
+５再生医療等製品の医療保険上の取扱いについて
+６費用対効果評価の結果を踏まえた薬価の見直しについて
+７DPCにおける高額な新規の医薬品等への対応について
+８在宅自己注射について
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第653回</t>
@@ -44,13 +68,6 @@
 ２再生医療等製品の保険適用について
 ３歯科用貴金属価格の随時改定について
 ４主な施設基準の届出状況等について
-</t>
-  </si>
-  <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
 </t>
   </si>
   <si>
@@ -846,7 +863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -920,7 +937,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -931,16 +948,16 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -960,7 +977,7 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -980,7 +997,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -1000,7 +1017,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -1020,7 +1037,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1040,7 +1057,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1060,7 +1077,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1080,7 +1097,7 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -1100,7 +1117,7 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1120,7 +1137,7 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1140,7 +1157,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -1160,7 +1177,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1180,7 +1197,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1200,7 +1217,7 @@
         <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1220,7 +1237,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1240,7 +1257,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1260,7 +1277,7 @@
         <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -1280,7 +1297,7 @@
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1300,7 +1317,7 @@
         <v>74</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1320,7 +1337,7 @@
         <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1340,7 +1357,7 @@
         <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1360,7 +1377,7 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1380,7 +1397,7 @@
         <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1400,7 +1417,7 @@
         <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1420,7 +1437,7 @@
         <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1440,7 +1457,7 @@
         <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -1460,7 +1477,7 @@
         <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -1480,7 +1497,7 @@
         <v>101</v>
       </c>
       <c r="D32" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -1500,7 +1517,7 @@
         <v>104</v>
       </c>
       <c r="D33" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -1520,7 +1537,7 @@
         <v>107</v>
       </c>
       <c r="D34" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -1540,12 +1557,32 @@
         <v>110</v>
       </c>
       <c r="D35" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
       </c>
       <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>111</v>
+      </c>
+      <c r="B36" t="s">
+        <v>112</v>
+      </c>
+      <c r="C36" t="s">
+        <v>113</v>
+      </c>
+      <c r="D36" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update num.txt | 2026-08-26 08:17:35 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="117">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,29 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第655回</t>
+  </si>
+  <si>
+    <t>2026年8月26日（令和8年8月26日）</t>
+  </si>
+  <si>
+    <t>１．費用対効果評価専門組_x000D_
+　　織からの報告について
+_x000D_
+２．ＯＴＣ類似薬の保険給_x000D_
+　　付の見直しについて
+_x000D_
+３．出産検討会の立ち上げ_x000D_
+　　について</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第654回</t>
@@ -51,13 +74,6 @@
 </t>
   </si>
   <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
-</t>
-  </si>
-  <si>
     <t>第653回</t>
   </si>
   <si>
@@ -68,6 +84,10 @@
 ２再生医療等製品の保険適用について
 ３歯科用貴金属価格の随時改定について
 ４主な施設基準の届出状況等について
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -100,10 +120,6 @@
 ５最適使用推進ガイドラインについて(報告)
 ６診療報酬改定結果検証部会からの報告について
 ７先進医療会議からの報告について
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -863,7 +879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -937,7 +953,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -948,16 +964,16 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -977,7 +993,7 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -997,7 +1013,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -1017,7 +1033,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -1037,7 +1053,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1057,7 +1073,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1077,7 +1093,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1097,7 +1113,7 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -1117,7 +1133,7 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1137,7 +1153,7 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1157,7 +1173,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -1177,7 +1193,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1197,7 +1213,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1217,7 +1233,7 @@
         <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1237,7 +1253,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1257,7 +1273,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1277,7 +1293,7 @@
         <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -1297,7 +1313,7 @@
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1317,7 +1333,7 @@
         <v>74</v>
       </c>
       <c r="D23" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1337,7 +1353,7 @@
         <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1357,7 +1373,7 @@
         <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1377,7 +1393,7 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1397,7 +1413,7 @@
         <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1417,7 +1433,7 @@
         <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1437,7 +1453,7 @@
         <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1457,7 +1473,7 @@
         <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -1477,7 +1493,7 @@
         <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -1497,7 +1513,7 @@
         <v>101</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -1517,7 +1533,7 @@
         <v>104</v>
       </c>
       <c r="D33" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -1537,7 +1553,7 @@
         <v>107</v>
       </c>
       <c r="D34" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -1557,7 +1573,7 @@
         <v>110</v>
       </c>
       <c r="D35" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -1577,12 +1593,32 @@
         <v>113</v>
       </c>
       <c r="D36" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
       </c>
       <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>114</v>
+      </c>
+      <c r="B37" t="s">
+        <v>115</v>
+      </c>
+      <c r="C37" t="s">
+        <v>116</v>
+      </c>
+      <c r="D37" t="s">
+        <v>17</v>
+      </c>
+      <c r="E37" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update num.txt | 2026-09-09 09:54:35 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="120">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,28 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第656回</t>
+  </si>
+  <si>
+    <t>2026年9月9日（令和8年9月9日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１最近の医療費の動向について
+２ＯＴＣ類似薬の保険給付の見直しについて（その２）
+３一部保険外療養の創設に伴う療養担当規則等の所要の見直しについて（諮問）
+４薬機法等改正に伴う保険薬局及び保険薬剤師療養担当規則等の所要の見直しについて（諮問）
+５個別改定項目について
+６その他
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第655回</t>
@@ -50,13 +72,6 @@
 　　について</t>
   </si>
   <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
-</t>
-  </si>
-  <si>
     <t>第654回</t>
   </si>
   <si>
@@ -74,6 +89,10 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">議事録
+</t>
+  </si>
+  <si>
     <t>第653回</t>
   </si>
   <si>
@@ -84,10 +103,6 @@
 ２再生医療等製品の保険適用について
 ３歯科用貴金属価格の随時改定について
 ４主な施設基準の届出状況等について
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -879,7 +894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1622,6 +1637,26 @@
         <v>9</v>
       </c>
     </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B38" t="s">
+        <v>118</v>
+      </c>
+      <c r="C38" t="s">
+        <v>119</v>
+      </c>
+      <c r="D38" t="s">
+        <v>17</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update num.txt | 2026-09-16 09:54:45 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="123">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,26 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第657回</t>
+  </si>
+  <si>
+    <t>2026年9月16日（令和8年9月16日）</t>
+  </si>
+  <si>
+    <t>１　 医療機器及び臨床検_x000D_
+　　 査の保険適用等につ_x000D_
+　　 いて_x000D_
+２　 個別改定項目につい_x000D_
+　　 て</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第656回</t>
@@ -45,14 +65,8 @@
 ３一部保険外療養の創設に伴う療養担当規則等の所要の見直しについて（諮問）
 ４薬機法等改正に伴う保険薬局及び保険薬剤師療養担当規則等の所要の見直しについて（諮問）
 ５個別改定項目について
-６その他
-</t>
-  </si>
-  <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
+６薬機法等改正に伴う保険薬局及び保険薬剤師療養担当規則等の所要の見直しについて（答申）
+７その他
 </t>
   </si>
   <si>
@@ -894,7 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -968,7 +982,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -979,16 +993,16 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -1008,7 +1022,7 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -1028,7 +1042,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -1048,7 +1062,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -1068,7 +1082,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1088,7 +1102,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1108,7 +1122,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1128,7 +1142,7 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -1148,7 +1162,7 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1168,7 +1182,7 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1188,7 +1202,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -1208,7 +1222,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1228,7 +1242,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1248,7 +1262,7 @@
         <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1268,7 +1282,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1288,7 +1302,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1308,7 +1322,7 @@
         <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -1328,7 +1342,7 @@
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1348,7 +1362,7 @@
         <v>74</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1368,7 +1382,7 @@
         <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1388,7 +1402,7 @@
         <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1408,7 +1422,7 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1428,7 +1442,7 @@
         <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1448,7 +1462,7 @@
         <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1468,7 +1482,7 @@
         <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1488,7 +1502,7 @@
         <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -1508,7 +1522,7 @@
         <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -1528,7 +1542,7 @@
         <v>101</v>
       </c>
       <c r="D32" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -1548,7 +1562,7 @@
         <v>104</v>
       </c>
       <c r="D33" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -1568,7 +1582,7 @@
         <v>107</v>
       </c>
       <c r="D34" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -1588,7 +1602,7 @@
         <v>110</v>
       </c>
       <c r="D35" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -1608,7 +1622,7 @@
         <v>113</v>
       </c>
       <c r="D36" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
@@ -1628,7 +1642,7 @@
         <v>116</v>
       </c>
       <c r="D37" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
@@ -1648,12 +1662,32 @@
         <v>119</v>
       </c>
       <c r="D38" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
       </c>
       <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>120</v>
+      </c>
+      <c r="B39" t="s">
+        <v>121</v>
+      </c>
+      <c r="C39" t="s">
+        <v>122</v>
+      </c>
+      <c r="D39" t="s">
+        <v>20</v>
+      </c>
+      <c r="E39" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update num.txt | 2026-09-30 10:45:54 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="126">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,31 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第658回</t>
+  </si>
+  <si>
+    <t>2026年9月30日（令和8年9月30日）</t>
+  </si>
+  <si>
+    <t>１　先進医療の科学的評価_x000D_
+　　結果についての報告
+２　最適使用推進ガイドラ_x000D_
+　　イン（簡略版）につい_x000D_
+　　て（審議）
+３　最適使用推進ガイドラ_x000D_
+　　インについて（報告）_x000D_
+４　公知申請とされた適応_x000D_
+　　外薬の保険適用につい_x000D_
+　　て</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第657回</t>
@@ -44,14 +69,8 @@
 　　 査の保険適用等につ_x000D_
 　　 いて_x000D_
 ２　 個別改定項目につい_x000D_
-　　 て</t>
-  </si>
-  <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
-</t>
+　　 て_x000D_
+３　 答申について</t>
   </si>
   <si>
     <t>第656回</t>
@@ -908,7 +927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1002,7 +1021,7 @@
         <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -1013,16 +1032,16 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -1042,7 +1061,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -1062,7 +1081,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -1082,7 +1101,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1102,7 +1121,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1122,7 +1141,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1142,7 +1161,7 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -1162,7 +1181,7 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1182,7 +1201,7 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1202,7 +1221,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -1222,7 +1241,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1242,7 +1261,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1262,7 +1281,7 @@
         <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1282,7 +1301,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1302,7 +1321,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1322,7 +1341,7 @@
         <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -1342,7 +1361,7 @@
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1362,7 +1381,7 @@
         <v>74</v>
       </c>
       <c r="D23" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1382,7 +1401,7 @@
         <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1402,7 +1421,7 @@
         <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1422,7 +1441,7 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1442,7 +1461,7 @@
         <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1462,7 +1481,7 @@
         <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1482,7 +1501,7 @@
         <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1502,7 +1521,7 @@
         <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -1522,7 +1541,7 @@
         <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -1542,7 +1561,7 @@
         <v>101</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -1562,7 +1581,7 @@
         <v>104</v>
       </c>
       <c r="D33" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -1582,7 +1601,7 @@
         <v>107</v>
       </c>
       <c r="D34" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -1602,7 +1621,7 @@
         <v>110</v>
       </c>
       <c r="D35" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -1622,7 +1641,7 @@
         <v>113</v>
       </c>
       <c r="D36" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
@@ -1642,7 +1661,7 @@
         <v>116</v>
       </c>
       <c r="D37" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
@@ -1662,7 +1681,7 @@
         <v>119</v>
       </c>
       <c r="D38" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
@@ -1682,12 +1701,32 @@
         <v>122</v>
       </c>
       <c r="D39" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
       </c>
       <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" t="s">
+        <v>125</v>
+      </c>
+      <c r="D40" t="s">
+        <v>23</v>
+      </c>
+      <c r="E40" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update num.txt | 2026-10-07 10:54:45 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="129">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,28 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第659回</t>
+  </si>
+  <si>
+    <t>2026年10月7日（令和8年10月7日）</t>
+  </si>
+  <si>
+    <t>１　医薬品の新規薬価収載_x000D_
+　　について_x000D_
+２　DPC における高額な_x000D_
+　　新規の医薬品等への_x000D_
+　　対応について_x000D_
+３　在宅自己注射について_x000D_
+４　その他</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第658回</t>
@@ -52,13 +74,6 @@
 　　て</t>
   </si>
   <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
-</t>
-  </si>
-  <si>
     <t>第657回</t>
   </si>
   <si>
@@ -105,6 +120,10 @@
 　　について</t>
   </si>
   <si>
+    <t xml:space="preserve">議事録
+</t>
+  </si>
+  <si>
     <t>第654回</t>
   </si>
   <si>
@@ -119,10 +138,6 @@
 ６費用対効果評価の結果を踏まえた薬価の見直しについて
 ７DPCにおける高額な新規の医薬品等への対応について
 ８在宅自己注射について
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -927,7 +942,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1730,6 +1745,26 @@
         <v>9</v>
       </c>
     </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>126</v>
+      </c>
+      <c r="B41" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" t="s">
+        <v>128</v>
+      </c>
+      <c r="D41" t="s">
+        <v>23</v>
+      </c>
+      <c r="E41" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>